<commit_message>
Update STEP2_Send_WhatsApp_v2.py with real @mention tagging and fixed group search
</commit_message>
<xml_diff>
--- a/DM contacts.xlsx
+++ b/DM contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anosha\Desktop\Reminder's Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E04EA272-89CF-4916-B452-9440AE377FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47619A46-30BD-4F66-8CEF-2FDE3CDDC931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9CA6DCC1-BFA5-43A1-AC84-92649301BE13}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$H$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="249">
   <si>
     <t>Market</t>
   </si>
@@ -156,12 +156,6 @@
     <t>DISTRICT MANAGER</t>
   </si>
   <si>
-    <t>MARKET MANAGER</t>
-  </si>
-  <si>
-    <t>HAMZA ALI</t>
-  </si>
-  <si>
     <t>bpe88706</t>
   </si>
   <si>
@@ -189,9 +183,6 @@
     <t>516-369-7846</t>
   </si>
   <si>
-    <t>NORTH CAROLINA</t>
-  </si>
-  <si>
     <t>qls25406</t>
   </si>
   <si>
@@ -255,9 +246,6 @@
     <t>(817) 448-5458</t>
   </si>
   <si>
-    <t>SHAIK MAZHAR UDDIN</t>
-  </si>
-  <si>
     <t>qev74584</t>
   </si>
   <si>
@@ -459,9 +447,6 @@
     <t>(214) 228-9687</t>
   </si>
   <si>
-    <t>ALI RIZVI</t>
-  </si>
-  <si>
     <t>lor29705</t>
   </si>
   <si>
@@ -471,9 +456,6 @@
     <t>919-259-6796</t>
   </si>
   <si>
-    <t>HASSAN TANVEER</t>
-  </si>
-  <si>
     <t>air06771</t>
   </si>
   <si>
@@ -483,9 +465,6 @@
     <t>347-888-2589</t>
   </si>
   <si>
-    <t>UZAIR UDDIN</t>
-  </si>
-  <si>
     <t>cxa39167</t>
   </si>
   <si>
@@ -504,12 +483,6 @@
     <t>(346) 758-1747</t>
   </si>
   <si>
-    <t>OXNARD/PALMDALE</t>
-  </si>
-  <si>
-    <t>ASLAM KHAN</t>
-  </si>
-  <si>
     <t>opk27999</t>
   </si>
   <si>
@@ -549,9 +522,6 @@
     <t>(901) 215-6410</t>
   </si>
   <si>
-    <t>TALHA QURESHI</t>
-  </si>
-  <si>
     <t>kdj61666</t>
   </si>
   <si>
@@ -597,123 +567,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>~Naqvi</t>
-  </si>
-  <si>
-    <t>~HAMED ALI SUFI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Anas </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~MA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Namir Mchantaf </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Farhan </t>
-  </si>
-  <si>
-    <t>~Abdullah</t>
-  </si>
-  <si>
-    <t>~Ahmed Imran</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Salim T </t>
-  </si>
-  <si>
-    <t>~Mazhar shaik</t>
-  </si>
-  <si>
-    <t>~Saad Ali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Haroon </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Ayan budhwani </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Sunvee </t>
-  </si>
-  <si>
-    <t>~Mukram</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Wajahat Ali </t>
-  </si>
-  <si>
-    <t>~Zubair Hussain</t>
-  </si>
-  <si>
-    <t>~SR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Maaz Z Khan </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Sharik </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Subhan Ansari </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Abdul Rafay </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Zaid </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Shoaib </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Amir </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Mr.Anas Ghory </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Sumair Farooqui </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Uzair </t>
-  </si>
-  <si>
-    <t>~Hassan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Ali Rizvi </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Ahmed Imran </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Prabha </t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Aslam Khan </t>
-  </si>
-  <si>
-    <t>~SRK</t>
-  </si>
-  <si>
-    <t>~Tee</t>
-  </si>
-  <si>
-    <t>~Asad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Hassan </t>
-  </si>
-  <si>
-    <t>~Kamran</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Nur Rahman </t>
-  </si>
-  <si>
     <t>OKLAHOMA</t>
   </si>
   <si>
@@ -723,9 +576,6 @@
     <t>Ayyan Budwani</t>
   </si>
   <si>
-    <t>~Ayyan Budwani</t>
-  </si>
-  <si>
     <t>Hamed Ali</t>
   </si>
   <si>
@@ -778,13 +628,172 @@
   </si>
   <si>
     <t>Merced &amp; Modesto</t>
+  </si>
+  <si>
+    <t>PHILY</t>
+  </si>
+  <si>
+    <t>HAMED ALI SUFI SYED</t>
+  </si>
+  <si>
+    <t>Muhammad Sumairuddin</t>
+  </si>
+  <si>
+    <t>+1 (214) 228-9687</t>
+  </si>
+  <si>
+    <t>Hassan Tanveer</t>
+  </si>
+  <si>
+    <t>SyedAli AhmedRizvi</t>
+  </si>
+  <si>
+    <t>Imran Shaikh</t>
+  </si>
+  <si>
+    <t>Uzair Uddin</t>
+  </si>
+  <si>
+    <t>Aslam Khan</t>
+  </si>
+  <si>
+    <t>Talha Qureshi</t>
+  </si>
+  <si>
+    <t>NORTH CAROL</t>
+  </si>
+  <si>
+    <t>Hamza Ali</t>
+  </si>
+  <si>
+    <t>OXNARD</t>
+  </si>
+  <si>
+    <t>PALMDALE</t>
+  </si>
+  <si>
+    <t>Naqvi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anas </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Namir Mchantaf </t>
+  </si>
+  <si>
+    <t>Abdullah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farhan </t>
+  </si>
+  <si>
+    <t>Ahmed Imran</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salim T </t>
+  </si>
+  <si>
+    <t>Mazhar shaik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ahmed Imran </t>
+  </si>
+  <si>
+    <t>Saad Ali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Haroon </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayan budhwani </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunvee </t>
+  </si>
+  <si>
+    <t>Mukarram</t>
+  </si>
+  <si>
+    <t>SR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wajahat Ali </t>
+  </si>
+  <si>
+    <t>Zubair Hussain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abdul Rafay </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maaz Z Khan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sharik </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subhan Ansari </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shoaib </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaid </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amir </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr.Anas Ghory </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sumair Farooqui </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ali Rizvi </t>
+  </si>
+  <si>
+    <t>Hassan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uzair </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prabha </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aslam Khan </t>
+  </si>
+  <si>
+    <t>SRK</t>
+  </si>
+  <si>
+    <t>HAMED ALI SUFI</t>
+  </si>
+  <si>
+    <t>Asad</t>
+  </si>
+  <si>
+    <t>Tee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hassan </t>
+  </si>
+  <si>
+    <t>Kamran</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nur Rahman </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -804,6 +813,17 @@
       <name val="Cambria"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -813,7 +833,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -821,11 +841,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -833,6 +868,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1148,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBC00CCB-5FAC-4DE4-8CA4-01E54F3D4AB5}">
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" bestFit="1" customWidth="1"/>
@@ -1166,7 +1213,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>230</v>
+        <v>180</v>
       </c>
       <c r="C1" t="s">
         <v>32</v>
@@ -1184,7 +1231,7 @@
         <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1192,25 +1239,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="C2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="D2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" t="s">
         <v>39</v>
       </c>
-      <c r="D2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>40</v>
       </c>
-      <c r="F2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2" t="s">
-        <v>42</v>
-      </c>
       <c r="H2" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1218,7 +1265,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>232</v>
+        <v>182</v>
       </c>
       <c r="C3" t="s">
         <v>2</v>
@@ -1227,16 +1274,16 @@
         <v>37</v>
       </c>
       <c r="E3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" t="s">
         <v>43</v>
       </c>
-      <c r="F3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" t="s">
-        <v>45</v>
-      </c>
       <c r="H3" t="s">
-        <v>185</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1247,19 +1294,19 @@
         <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" t="s">
         <v>46</v>
       </c>
-      <c r="F4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" t="s">
-        <v>48</v>
-      </c>
       <c r="H4" t="s">
-        <v>187</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1270,19 +1317,19 @@
         <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="H5" t="s">
-        <v>188</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1296,16 +1343,16 @@
         <v>37</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H6" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1313,25 +1360,25 @@
         <v>9</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>232</v>
+        <v>182</v>
       </c>
       <c r="C7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" t="s">
         <v>56</v>
       </c>
-      <c r="D7" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" t="s">
-        <v>58</v>
-      </c>
-      <c r="G7" t="s">
-        <v>59</v>
-      </c>
       <c r="H7" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1339,7 +1386,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>233</v>
+        <v>183</v>
       </c>
       <c r="C8" t="s">
         <v>10</v>
@@ -1348,16 +1395,16 @@
         <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H8" t="s">
-        <v>190</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1365,22 +1412,22 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" t="s">
         <v>63</v>
       </c>
-      <c r="D9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" t="s">
-        <v>64</v>
-      </c>
-      <c r="F9" t="s">
-        <v>65</v>
-      </c>
-      <c r="G9" t="s">
-        <v>66</v>
-      </c>
       <c r="H9" t="s">
-        <v>192</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1388,68 +1435,68 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" t="s">
         <v>67</v>
       </c>
-      <c r="D10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" t="s">
-        <v>68</v>
-      </c>
-      <c r="F10" t="s">
-        <v>69</v>
-      </c>
-      <c r="G10" t="s">
-        <v>70</v>
-      </c>
       <c r="H10" t="s">
-        <v>193</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="C11" t="s">
-        <v>71</v>
+      <c r="C11" s="4" t="s">
+        <v>202</v>
       </c>
       <c r="D11" t="s">
         <v>37</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G11" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H11" t="s">
-        <v>194</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>224</v>
+        <v>175</v>
       </c>
       <c r="C12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" t="s">
         <v>63</v>
       </c>
-      <c r="D12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12" t="s">
-        <v>64</v>
-      </c>
-      <c r="F12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G12" t="s">
-        <v>66</v>
-      </c>
       <c r="H12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1457,25 +1504,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>234</v>
+        <v>184</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E13" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F13" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G13" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H13" t="s">
-        <v>195</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1483,22 +1530,22 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E14" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G14" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H14" t="s">
-        <v>196</v>
+        <v>221</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1506,22 +1553,22 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G15" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H15" t="s">
-        <v>197</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1529,7 +1576,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>232</v>
+        <v>182</v>
       </c>
       <c r="C16" t="s">
         <v>16</v>
@@ -1538,16 +1585,16 @@
         <v>37</v>
       </c>
       <c r="E16" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F16" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G16" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H16" t="s">
-        <v>198</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1555,7 +1602,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>235</v>
+        <v>185</v>
       </c>
       <c r="C17" t="s">
         <v>17</v>
@@ -1564,16 +1611,16 @@
         <v>37</v>
       </c>
       <c r="E17" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G17" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H17" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1581,25 +1628,25 @@
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>233</v>
+        <v>183</v>
       </c>
       <c r="C18" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
       </c>
       <c r="E18" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F18" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G18" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="H18" t="s">
-        <v>202</v>
+        <v>225</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1607,7 +1654,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>231</v>
+        <v>181</v>
       </c>
       <c r="C19" t="s">
         <v>18</v>
@@ -1616,16 +1663,16 @@
         <v>37</v>
       </c>
       <c r="E19" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F19" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G19" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="H19" t="s">
-        <v>200</v>
+        <v>226</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1633,25 +1680,25 @@
         <v>15</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>236</v>
+        <v>186</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D20" t="s">
         <v>37</v>
       </c>
       <c r="E20" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F20" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="G20" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H20" t="s">
-        <v>201</v>
+        <v>227</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1659,25 +1706,25 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>237</v>
+        <v>187</v>
       </c>
       <c r="C21" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E21" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F21" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G21" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H21" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1685,25 +1732,25 @@
         <v>20</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>238</v>
+        <v>188</v>
       </c>
       <c r="C22" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E22" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F22" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G22" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H22" t="s">
-        <v>203</v>
+        <v>229</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1711,25 +1758,25 @@
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>239</v>
+        <v>189</v>
       </c>
       <c r="C23" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F23" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G23" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="H23" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1737,25 +1784,25 @@
         <v>20</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="C24" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E24" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F24" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G24" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H24" t="s">
-        <v>205</v>
+        <v>231</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1763,22 +1810,22 @@
         <v>21</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D25" t="s">
         <v>37</v>
       </c>
       <c r="E25" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F25" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G25" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H25" t="s">
-        <v>208</v>
+        <v>232</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1786,25 +1833,25 @@
         <v>21</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>232</v>
+        <v>182</v>
       </c>
       <c r="C26" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D26" t="s">
         <v>37</v>
       </c>
       <c r="E26" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G26" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="H26" t="s">
-        <v>207</v>
+        <v>233</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1812,45 +1859,45 @@
         <v>21</v>
       </c>
       <c r="C27" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D27" t="s">
         <v>37</v>
       </c>
       <c r="E27" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F27" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="G27" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="H27" t="s">
-        <v>209</v>
+        <v>234</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>225</v>
+        <v>176</v>
       </c>
       <c r="C28" t="s">
         <v>19</v>
       </c>
       <c r="D28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E28" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F28" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="G28" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H28" t="s">
-        <v>210</v>
+        <v>235</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1858,97 +1905,97 @@
         <v>22</v>
       </c>
       <c r="C29" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E29" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F29" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="G29" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H29" t="s">
-        <v>211</v>
+        <v>236</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>49</v>
-      </c>
-      <c r="C30" t="s">
-        <v>139</v>
+        <v>206</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>201</v>
       </c>
       <c r="D30" t="s">
         <v>37</v>
       </c>
       <c r="E30" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F30" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G30" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="H30" t="s">
-        <v>214</v>
+        <v>237</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>49</v>
+        <v>206</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="C31" t="s">
-        <v>143</v>
+        <v>191</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>200</v>
       </c>
       <c r="D31" t="s">
         <v>37</v>
       </c>
       <c r="E31" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="F31" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G31" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="H31" t="s">
-        <v>213</v>
+        <v>238</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>49</v>
+        <v>206</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="C32" t="s">
-        <v>147</v>
+        <v>192</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>203</v>
       </c>
       <c r="D32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E32" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="F32" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="G32" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="H32" t="s">
-        <v>212</v>
+        <v>239</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -1959,120 +2006,120 @@
         <v>24</v>
       </c>
       <c r="D33" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E33" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="F33" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G33" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="H33" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>154</v>
+      <c r="A34" s="6" t="s">
+        <v>209</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="C34" t="s">
-        <v>155</v>
+        <v>193</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="D34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E34" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="F34" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="G34" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="H34" t="s">
-        <v>217</v>
+        <v>241</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>25</v>
-      </c>
-      <c r="C35" t="s">
-        <v>26</v>
+      <c r="A35" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="D35" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E35" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="F35" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="G35" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="H35" t="s">
-        <v>218</v>
+        <v>241</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>1</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>236</v>
+        <v>25</v>
       </c>
       <c r="C36" t="s">
-        <v>228</v>
+        <v>26</v>
       </c>
       <c r="D36" t="s">
         <v>37</v>
       </c>
       <c r="E36" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="F36" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="G36" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="H36" t="s">
-        <v>186</v>
+        <v>242</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>244</v>
+        <v>186</v>
       </c>
       <c r="C37" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D37" t="s">
         <v>37</v>
       </c>
       <c r="E37" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="F37" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="G37" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="H37" t="s">
-        <v>220</v>
+        <v>243</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -2080,117 +2127,183 @@
         <v>27</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>245</v>
+        <v>194</v>
       </c>
       <c r="C38" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="D38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E38" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="F38" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="G38" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="H38" t="s">
-        <v>219</v>
+        <v>244</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>28</v>
-      </c>
-      <c r="C39" t="s">
-        <v>173</v>
+        <v>27</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>205</v>
       </c>
       <c r="D39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E39" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="F39" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="G39" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="H39" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C40" t="s">
-        <v>229</v>
+        <v>163</v>
       </c>
       <c r="D40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E40" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="F40" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="G40" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="H40" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C41" t="s">
-        <v>31</v>
+        <v>179</v>
       </c>
       <c r="D41" t="s">
         <v>37</v>
       </c>
       <c r="E41" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="F41" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="G41" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="H41" t="s">
-        <v>223</v>
+        <v>247</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" t="s">
+        <v>31</v>
+      </c>
+      <c r="D42" t="s">
+        <v>37</v>
+      </c>
+      <c r="E42" t="s">
+        <v>170</v>
+      </c>
+      <c r="F42" t="s">
+        <v>171</v>
+      </c>
+      <c r="G42" t="s">
+        <v>172</v>
+      </c>
+      <c r="H42" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>14</v>
       </c>
-      <c r="C42" t="s">
-        <v>226</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>227</v>
+      <c r="C43" t="s">
+        <v>177</v>
+      </c>
+      <c r="D43" t="s">
+        <v>37</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>196</v>
+      </c>
+      <c r="C44" t="s">
+        <v>197</v>
+      </c>
+      <c r="D44" t="s">
+        <v>37</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H44" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D45" t="s">
+        <v>37</v>
+      </c>
+      <c r="G45" t="s">
+        <v>199</v>
+      </c>
+      <c r="H45" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tagging problem was resolved
</commit_message>
<xml_diff>
--- a/DM contacts.xlsx
+++ b/DM contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anosha\Desktop\Reminder's Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47619A46-30BD-4F66-8CEF-2FDE3CDDC931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49921ED3-EB18-404B-A999-8B3F0EA6460E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9CA6DCC1-BFA5-43A1-AC84-92649301BE13}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="248">
   <si>
     <t>Market</t>
   </si>
@@ -681,36 +681,18 @@
     <t xml:space="preserve">MA </t>
   </si>
   <si>
-    <t xml:space="preserve">Namir Mchantaf </t>
-  </si>
-  <si>
     <t>Abdullah</t>
   </si>
   <si>
     <t xml:space="preserve">Farhan </t>
   </si>
   <si>
-    <t>Ahmed Imran</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salim T </t>
-  </si>
-  <si>
     <t>Mazhar shaik</t>
   </si>
   <si>
-    <t xml:space="preserve">Ahmed Imran </t>
-  </si>
-  <si>
-    <t>Saad Ali</t>
-  </si>
-  <si>
     <t xml:space="preserve">Haroon </t>
   </si>
   <si>
-    <t xml:space="preserve">Ayan budhwani </t>
-  </si>
-  <si>
     <t xml:space="preserve">Sunvee </t>
   </si>
   <si>
@@ -720,24 +702,9 @@
     <t>SR</t>
   </si>
   <si>
-    <t xml:space="preserve">Wajahat Ali </t>
-  </si>
-  <si>
-    <t>Zubair Hussain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abdul Rafay </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maaz Z Khan </t>
-  </si>
-  <si>
     <t xml:space="preserve">Sharik </t>
   </si>
   <si>
-    <t xml:space="preserve">Subhan Ansari </t>
-  </si>
-  <si>
     <t xml:space="preserve">Shoaib </t>
   </si>
   <si>
@@ -747,15 +714,6 @@
     <t xml:space="preserve">Amir </t>
   </si>
   <si>
-    <t xml:space="preserve">Mr.Anas Ghory </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sumair Farooqui </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ali Rizvi </t>
-  </si>
-  <si>
     <t>Hassan</t>
   </si>
   <si>
@@ -765,15 +723,9 @@
     <t xml:space="preserve">Prabha </t>
   </si>
   <si>
-    <t xml:space="preserve">Aslam Khan </t>
-  </si>
-  <si>
     <t>SRK</t>
   </si>
   <si>
-    <t>HAMED ALI SUFI</t>
-  </si>
-  <si>
     <t>Asad</t>
   </si>
   <si>
@@ -786,7 +738,52 @@
     <t>Kamran</t>
   </si>
   <si>
-    <t xml:space="preserve">Nur Rahman </t>
+    <t>Namir</t>
+  </si>
+  <si>
+    <t>Ahmed</t>
+  </si>
+  <si>
+    <t>Salim</t>
+  </si>
+  <si>
+    <t>Saad</t>
+  </si>
+  <si>
+    <t>Ayan</t>
+  </si>
+  <si>
+    <t>Wajahat</t>
+  </si>
+  <si>
+    <t>Zubair</t>
+  </si>
+  <si>
+    <t>Abdul</t>
+  </si>
+  <si>
+    <t>Maaz</t>
+  </si>
+  <si>
+    <t>Subhan</t>
+  </si>
+  <si>
+    <t>Mr.Anas</t>
+  </si>
+  <si>
+    <t>Sumair</t>
+  </si>
+  <si>
+    <t>Ali</t>
+  </si>
+  <si>
+    <t>Aslam</t>
+  </si>
+  <si>
+    <t>HAMED</t>
+  </si>
+  <si>
+    <t>Nur</t>
   </si>
 </sst>
 </file>
@@ -1352,7 +1349,7 @@
         <v>52</v>
       </c>
       <c r="H6" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1378,7 +1375,7 @@
         <v>56</v>
       </c>
       <c r="H7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1404,7 +1401,7 @@
         <v>59</v>
       </c>
       <c r="H8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1427,7 +1424,7 @@
         <v>63</v>
       </c>
       <c r="H9" t="s">
-        <v>216</v>
+        <v>233</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1450,7 +1447,7 @@
         <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>217</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1473,7 +1470,7 @@
         <v>70</v>
       </c>
       <c r="H11" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1496,7 +1493,7 @@
         <v>63</v>
       </c>
       <c r="H12" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1522,7 +1519,7 @@
         <v>74</v>
       </c>
       <c r="H13" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1545,7 +1542,7 @@
         <v>78</v>
       </c>
       <c r="H14" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1568,7 +1565,7 @@
         <v>82</v>
       </c>
       <c r="H15" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1594,7 +1591,7 @@
         <v>85</v>
       </c>
       <c r="H16" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1620,7 +1617,7 @@
         <v>88</v>
       </c>
       <c r="H17" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1646,7 +1643,7 @@
         <v>92</v>
       </c>
       <c r="H18" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1672,7 +1669,7 @@
         <v>95</v>
       </c>
       <c r="H19" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1698,7 +1695,7 @@
         <v>99</v>
       </c>
       <c r="H20" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1724,7 +1721,7 @@
         <v>103</v>
       </c>
       <c r="H21" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1750,7 +1747,7 @@
         <v>107</v>
       </c>
       <c r="H22" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1776,7 +1773,7 @@
         <v>111</v>
       </c>
       <c r="H23" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1802,7 +1799,7 @@
         <v>115</v>
       </c>
       <c r="H24" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1825,7 +1822,7 @@
         <v>119</v>
       </c>
       <c r="H25" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1851,7 +1848,7 @@
         <v>123</v>
       </c>
       <c r="H26" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1874,7 +1871,7 @@
         <v>127</v>
       </c>
       <c r="H27" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -1897,7 +1894,7 @@
         <v>130</v>
       </c>
       <c r="H28" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1920,7 +1917,7 @@
         <v>134</v>
       </c>
       <c r="H29" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1943,7 +1940,7 @@
         <v>137</v>
       </c>
       <c r="H30" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -1969,7 +1966,7 @@
         <v>140</v>
       </c>
       <c r="H31" t="s">
-        <v>238</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1995,7 +1992,7 @@
         <v>143</v>
       </c>
       <c r="H32" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -2018,7 +2015,7 @@
         <v>146</v>
       </c>
       <c r="H33" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -2044,7 +2041,7 @@
         <v>149</v>
       </c>
       <c r="H34" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -2070,7 +2067,7 @@
         <v>149</v>
       </c>
       <c r="H35" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -2093,7 +2090,7 @@
         <v>152</v>
       </c>
       <c r="H36" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -2119,7 +2116,7 @@
         <v>155</v>
       </c>
       <c r="H37" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -2145,7 +2142,7 @@
         <v>159</v>
       </c>
       <c r="H38" t="s">
-        <v>244</v>
+        <v>228</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -2171,7 +2168,7 @@
         <v>162</v>
       </c>
       <c r="H39" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -2194,7 +2191,7 @@
         <v>166</v>
       </c>
       <c r="H40" t="s">
-        <v>246</v>
+        <v>230</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -2217,7 +2214,7 @@
         <v>169</v>
       </c>
       <c r="H41" t="s">
-        <v>247</v>
+        <v>231</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -2240,7 +2237,7 @@
         <v>172</v>
       </c>
       <c r="H42" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -2263,7 +2260,7 @@
         <v>82</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>177</v>
+        <v>236</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2286,7 +2283,7 @@
         <v>155</v>
       </c>
       <c r="H44" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2303,7 +2300,7 @@
         <v>199</v>
       </c>
       <c r="H45" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>